<commit_message>
Big Update - Full deployment Phase 5A
</commit_message>
<xml_diff>
--- a/app/Data/accumulation/Aichi_Accumulated.xlsx
+++ b/app/Data/accumulation/Aichi_Accumulated.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記入例" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="English ver 記入例" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年1月" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追加1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年2月" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年3月" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年4月" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年5月" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年6月" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年7月" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年8月" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年9月" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年10月" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年11月" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年12月" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="集計ﾃｰﾌﾞﾙ" sheetId="16" state="hidden" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024年11月" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年07月" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024年12月" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="記入例" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="English ver 記入例" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025年1月" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="追加1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2025年2月" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2025年3月" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2025年4月" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2025年5月" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2025年6月" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2025年7月" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2025年8月" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2025年9月" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2025年10月" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2025年11月" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2025年12月" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="集計ﾃｰﾌﾞﾙ" sheetId="16" state="hidden" r:id="rId16"/>
+    <sheet name="2024年11月" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2025年07月" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2024年12月" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="ExternalData_4" localSheetId="3">'追加1'!$A$1:$H$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="0" r:id="rId20"/>
+    <pivotCache cacheId="0" r:id="rId20"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -18475,7 +18475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X45"/>
+  <dimension ref="A1:X47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="9" customWidth="1" style="115" min="1" max="1"/>
@@ -18683,7 +18683,7 @@
       </c>
       <c r="U5" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
     </row>
@@ -19480,7 +19480,7 @@
       </c>
       <c r="U17" s="104" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="V17" s="104" t="n"/>
@@ -20694,8 +20694,106 @@
         <v>250</v>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1" s="115"/>
-    <row r="47" ht="18" customHeight="1" s="115"/>
+    <row r="46" ht="18" customHeight="1" s="115">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2024-11-20</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="inlineStr"/>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Test Vendor 株式会社</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Ethan Cole</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr"/>
+      <c r="F46" s="0" t="n">
+        <v>12345</v>
+      </c>
+      <c r="G46" s="0" t="inlineStr"/>
+      <c r="H46" s="0" t="inlineStr">
+        <is>
+          <t>TEST-INVOICE-1768717972</t>
+        </is>
+      </c>
+      <c r="I46" s="0" t="inlineStr"/>
+      <c r="J46" s="0" t="inlineStr"/>
+      <c r="K46" s="0" t="n">
+        <v>1234</v>
+      </c>
+      <c r="L46" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" s="0" t="inlineStr"/>
+      <c r="N46" s="0" t="n">
+        <v>12345</v>
+      </c>
+      <c r="O46" s="0" t="inlineStr"/>
+      <c r="P46" s="0" t="n">
+        <v>1234</v>
+      </c>
+      <c r="Q46" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" s="0" t="n">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="115">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2024-11-20</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Test Vendor 株式会社</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Ethan Cole</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>12345</v>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>TEST-INVOICE-1768717972</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="n">
+        <v>1234</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="n">
+        <v>12345</v>
+      </c>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="n">
+        <v>1234</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" t="n">
+        <v>1234</v>
+      </c>
+    </row>
     <row r="48" ht="18" customHeight="1" s="115"/>
     <row r="49" ht="18" customHeight="1" s="115"/>
     <row r="50" ht="18" customHeight="1" s="115"/>
@@ -21877,7 +21975,7 @@
       </c>
       <c r="U5" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
     </row>
@@ -22674,7 +22772,7 @@
       </c>
       <c r="U17" s="104" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="V17" s="104" t="n"/>
@@ -24887,7 +24985,7 @@
       </c>
       <c r="U5" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
     </row>
@@ -25684,7 +25782,7 @@
       </c>
       <c r="U17" s="104" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="V17" s="104" t="n"/>
@@ -26661,52 +26759,52 @@
       <c r="R40" s="45" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1" s="115">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
         <is>
           <t>2024-12-10</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr"/>
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>Uny OiI</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>Lucas Bennett</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="n">
+      <c r="E41" s="0" t="inlineStr"/>
+      <c r="F41" s="0" t="n">
         <v>5000</v>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
+      <c r="G41" s="0" t="inlineStr"/>
+      <c r="H41" s="0" t="inlineStr">
         <is>
           <t>T2180001091960</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="n">
+      <c r="I41" s="0" t="inlineStr"/>
+      <c r="J41" s="0" t="inlineStr"/>
+      <c r="K41" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="L41" t="n">
+      <c r="L41" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="n">
+      <c r="M41" s="0" t="inlineStr"/>
+      <c r="N41" s="0" t="n">
         <v>5000</v>
       </c>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="n">
+      <c r="O41" s="0" t="inlineStr"/>
+      <c r="P41" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="Q41" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="R41" t="n">
+      <c r="R41" s="0" t="n">
         <v>3</v>
       </c>
     </row>
@@ -30246,7 +30344,7 @@
       </c>
       <c r="U5" s="100" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
     </row>
@@ -31043,7 +31141,7 @@
       </c>
       <c r="U17" s="104" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="V17" s="104" t="n"/>

</xml_diff>